<commit_message>
fix(elearning-laporan): kolom hari/tanggal agenda tutor diambil dari waktu tutor pertama isi daftar hadir, bukan startDate
</commit_message>
<xml_diff>
--- a/public/templates/format-upload-pengelola.xlsx
+++ b/public/templates/format-upload-pengelola.xlsx
@@ -44,10 +44,10 @@
     <t>Agama</t>
   </si>
   <si>
+    <t>Pendidikan Terakhir</t>
+  </si>
+  <si>
     <t>Alamat</t>
-  </si>
-  <si>
-    <t>Pendidikan Terakhir</t>
   </si>
   <si>
     <t>RT</t>
@@ -532,17 +532,17 @@
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.71094" customWidth="1"/>
     <col min="8" max="8" width="7.710938" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9" customWidth="1"/>
+    <col min="9" max="9" width="12.57031" customWidth="1"/>
+    <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.425781" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="5.570313" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="4.425781" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.570313" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" customWidth="1"/>
-    <col min="16" max="16" width="13.28516" customWidth="1"/>
-    <col min="17" max="17" width="10.42578" customWidth="1"/>
-    <col min="18" max="18" width="20.71094" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.570313" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.85547" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.71094" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.855469" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="3.710938" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.28516" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="14" customWidth="1"/>
     <col min="21" max="21" width="16" customWidth="1"/>
     <col min="22" max="22" width="14.14063" customWidth="1"/>
@@ -576,63 +576,61 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" s="3" t="s">
         <v>25</v>
       </c>
+      <c r="AA1"/>
     </row>
     <row r="2">
       <c r="A2" s="4"/>
@@ -661,7 +659,7 @@
       <c r="X2" s="4"/>
       <c r="Y2" s="4"/>
       <c r="Z2" s="4"/>
-      <c r="AA2" s="4"/>
+      <c r="AA2"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>